<commit_message>
Update logs and reports for retorno-ligacoes-oficial and ercard-tabela-contratos processes
- Adjusted timestamps and durations in agente_estado.json, agente_relatorio_final.json, and agente_historico.jsonl for the retorno-ligacoes-oficial process.
- Added new entries for ercard-tabela-contratos in agente_historico.jsonl, including error handling for a failed attempt.
- Updated ercard_carteira_estado.json to reflect the latest execution details and errors encountered during the process.
- Modified ercard_tabela_contratos_estado.json to include error messages related to session issues.
- Revised relatorio_validacao.json to reflect changes in validation status and errors found in the migration files.
- Added new log file for agendado_ercard_carteira with detailed execution steps and errors.
- Updated binary file fat_metas_venda_moda_lojas_hoje.xlsx to reflect new data.
</commit_message>
<xml_diff>
--- a/CREDIAGORA/teste_migracao_oficiais/fat_metas_venda_moda_lojas_hoje.xlsx
+++ b/CREDIAGORA/teste_migracao_oficiais/fat_metas_venda_moda_lojas_hoje.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tjipromotora.sharepoint.com/sites/Crediagora-doc/Data Science/dados/tabela fat/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CREDIAGORA\Desktop\workspace\Automacoes\crediagora\CREDIAGORA\teste_migracao_oficiais\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8407" documentId="13_ncr:1_{B332BB96-64E4-4EF7-B5A3-C0F398143B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF612464-2CA3-4A0F-ADD0-969E1E3E74E0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B00864-D7F3-402C-8D11-82E45F8A2664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{8E47A5CF-CF99-4C53-84E9-B0BB5F4D1E77}"/>
+    <workbookView xWindow="5316" yWindow="4056" windowWidth="13836" windowHeight="7968" xr2:uid="{8E47A5CF-CF99-4C53-84E9-B0BB5F4D1E77}"/>
   </bookViews>
   <sheets>
     <sheet name="base" sheetId="1" r:id="rId1"/>
@@ -1993,10 +1993,12 @@
         <f>L3</f>
         <v>7213.78</v>
       </c>
-      <c r="C18" s="16"/>
+      <c r="C18" s="16">
+        <v>1968.84</v>
+      </c>
       <c r="D18" s="28">
         <f>C18/B18</f>
-        <v>0</v>
+        <v>0.27292764680930109</v>
       </c>
       <c r="E18" s="30">
         <f>'[1]P Eliane'!$I$3</f>
@@ -2008,7 +2010,7 @@
       </c>
       <c r="G18" s="30">
         <f t="shared" ref="G18:G26" si="1">SUM(F18,C18)</f>
-        <v>1790.88</v>
+        <v>3759.7200000000003</v>
       </c>
       <c r="H18" s="8"/>
       <c r="J18" s="6"/>
@@ -2023,10 +2025,12 @@
         <f>L7</f>
         <v>7065.22</v>
       </c>
-      <c r="C19" s="16"/>
+      <c r="C19" s="16">
+        <v>2812.71</v>
+      </c>
       <c r="D19" s="28">
         <f t="shared" ref="D19:D25" si="2">C19/B19</f>
-        <v>0</v>
+        <v>0.3981064991606772</v>
       </c>
       <c r="E19" s="30">
         <f>'[1]P Eliane'!$I$7</f>
@@ -2038,7 +2042,7 @@
       </c>
       <c r="G19" s="30">
         <f t="shared" si="1"/>
-        <v>399.96</v>
+        <v>3212.67</v>
       </c>
       <c r="H19" s="8"/>
       <c r="J19" s="6"/>
@@ -2053,10 +2057,12 @@
         <f>L8</f>
         <v>7008.11</v>
       </c>
-      <c r="C20" s="16"/>
+      <c r="C20" s="16">
+        <v>2156.61</v>
+      </c>
       <c r="D20" s="28">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.30773061495895471</v>
       </c>
       <c r="E20" s="30">
         <f>'[1]P Eliane'!$I$8</f>
@@ -2068,7 +2074,7 @@
       </c>
       <c r="G20" s="30">
         <f t="shared" si="1"/>
-        <v>1280.4000000000001</v>
+        <v>3437.01</v>
       </c>
       <c r="H20" s="8"/>
       <c r="J20" s="6"/>
@@ -2083,10 +2089,12 @@
         <f>L9</f>
         <v>8318.49</v>
       </c>
-      <c r="C21" s="16"/>
+      <c r="C21" s="16">
+        <v>4765.3900000000003</v>
+      </c>
       <c r="D21" s="28">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.57286719104068173</v>
       </c>
       <c r="E21" s="30">
         <f>'[1]P Eliane'!$I$9</f>
@@ -2098,7 +2106,7 @@
       </c>
       <c r="G21" s="30">
         <f t="shared" si="1"/>
-        <v>2584.08</v>
+        <v>7349.47</v>
       </c>
       <c r="H21" s="8"/>
       <c r="J21" s="6"/>
@@ -2113,10 +2121,12 @@
         <f>L5</f>
         <v>6035.68</v>
       </c>
-      <c r="C22" s="16"/>
+      <c r="C22" s="16">
+        <v>3045.48</v>
+      </c>
       <c r="D22" s="28">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.50457943429737828</v>
       </c>
       <c r="E22" s="30">
         <f>'[1]P Eliane'!$I$5</f>
@@ -2128,7 +2138,7 @@
       </c>
       <c r="G22" s="30">
         <f t="shared" si="1"/>
-        <v>1573.08</v>
+        <v>4618.5599999999995</v>
       </c>
       <c r="H22" s="8"/>
       <c r="J22" s="6"/>
@@ -2143,10 +2153,12 @@
         <f>L6</f>
         <v>7485.78</v>
       </c>
-      <c r="C23" s="16"/>
+      <c r="C23" s="16">
+        <v>6491.14</v>
+      </c>
       <c r="D23" s="28">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.86712941069601301</v>
       </c>
       <c r="E23" s="30">
         <f>'[1]P Eliane'!$I$6</f>
@@ -2158,7 +2170,7 @@
       </c>
       <c r="G23" s="30">
         <f t="shared" si="1"/>
-        <v>1912.32</v>
+        <v>8403.4600000000009</v>
       </c>
       <c r="H23" s="8"/>
       <c r="J23" s="6"/>
@@ -2173,10 +2185,12 @@
         <f>L4</f>
         <v>8089.69</v>
       </c>
-      <c r="C24" s="16"/>
+      <c r="C24" s="16">
+        <v>1681.05</v>
+      </c>
       <c r="D24" s="28">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.20780153504027968</v>
       </c>
       <c r="E24" s="30">
         <f>'[1]P Eliane'!$I$4</f>
@@ -2188,7 +2202,7 @@
       </c>
       <c r="G24" s="30">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1681.05</v>
       </c>
       <c r="H24" s="8"/>
       <c r="J24" s="6"/>
@@ -2203,10 +2217,12 @@
         <f>L2</f>
         <v>7092.06</v>
       </c>
-      <c r="C25" s="16"/>
+      <c r="C25" s="16">
+        <v>4478.92</v>
+      </c>
       <c r="D25" s="28">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.63154006029277809</v>
       </c>
       <c r="E25" s="30">
         <f>'[1]P Eliane'!$I$2</f>
@@ -2218,7 +2234,7 @@
       </c>
       <c r="G25" s="30">
         <f t="shared" si="1"/>
-        <v>426.6</v>
+        <v>4905.5200000000004</v>
       </c>
       <c r="H25" s="8"/>
       <c r="J25" s="6"/>
@@ -2257,11 +2273,11 @@
       </c>
       <c r="C27" s="14">
         <f>SUM(C18:C25)</f>
-        <v>0</v>
+        <v>27400.14</v>
       </c>
       <c r="D27" s="29">
         <f>C27/B27</f>
-        <v>0</v>
+        <v>0.4699142376597979</v>
       </c>
       <c r="E27" s="38">
         <f>SUM(E18:E25)</f>
@@ -2273,7 +2289,7 @@
       </c>
       <c r="G27" s="31">
         <f>SUM(G18:G25)</f>
-        <v>9967.32</v>
+        <v>37367.46</v>
       </c>
       <c r="H27" s="8"/>
       <c r="J27" s="6"/>
@@ -2303,11 +2319,11 @@
       </c>
       <c r="C29" s="14">
         <f>C27+F10</f>
-        <v>450603.14999999997</v>
+        <v>478003.29</v>
       </c>
       <c r="D29" s="15">
         <f>C29/B29</f>
-        <v>0.41264024725274723</v>
+        <v>0.43773195054945052</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
@@ -2770,15 +2786,15 @@
       </c>
       <c r="C2" s="10">
         <f>base!C27</f>
-        <v>0</v>
+        <v>27400.14</v>
       </c>
       <c r="D2" s="8">
         <f>IFERROR(C2/B2,0)</f>
-        <v>0</v>
+        <v>0.4699142376597979</v>
       </c>
       <c r="E2" s="7">
         <f>B2-C2</f>
-        <v>58308.81</v>
+        <v>30908.67</v>
       </c>
       <c r="F2" s="11">
         <f>base!F11-base!D11</f>
@@ -2849,26 +2865,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="671776c5-29b2-438f-93e2-4095a3782164" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fb12f9d3-8460-4672-9bb3-c98df481edea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E2BA6437EF849047B33977AE3CC00025" ma:contentTypeVersion="15" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="2fda3b91f0fc8e20c14c11d32d8864dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="671776c5-29b2-438f-93e2-4095a3782164" xmlns:ns3="fb12f9d3-8460-4672-9bb3-c98df481edea" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="161cc5a8399f8fd96cc67feff6bac404" ns2:_="" ns3:_="">
     <xsd:import namespace="671776c5-29b2-438f-93e2-4095a3782164"/>
@@ -3103,10 +3099,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="671776c5-29b2-438f-93e2-4095a3782164" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fb12f9d3-8460-4672-9bb3-c98df481edea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{073DE036-2C71-4DAE-AACC-05156901298A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADD69931-4CC0-4D4D-BBD5-76BF95E19BCA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="671776c5-29b2-438f-93e2-4095a3782164"/>
+    <ds:schemaRef ds:uri="fb12f9d3-8460-4672-9bb3-c98df481edea"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3129,20 +3156,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADD69931-4CC0-4D4D-BBD5-76BF95E19BCA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{073DE036-2C71-4DAE-AACC-05156901298A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="671776c5-29b2-438f-93e2-4095a3782164"/>
-    <ds:schemaRef ds:uri="fb12f9d3-8460-4672-9bb3-c98df481edea"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
atualização de arquivos Excel de migração
</commit_message>
<xml_diff>
--- a/CREDIAGORA/teste_migracao_oficiais/fat_metas_venda_moda_lojas_hoje.xlsx
+++ b/CREDIAGORA/teste_migracao_oficiais/fat_metas_venda_moda_lojas_hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CREDIAGORA\Desktop\workspace\Automacoes\crediagora\CREDIAGORA\teste_migracao_oficiais\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B00864-D7F3-402C-8D11-82E45F8A2664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B5B9DB3-074A-4854-A497-DFD73CF72154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5316" yWindow="4056" windowWidth="13836" windowHeight="7968" xr2:uid="{8E47A5CF-CF99-4C53-84E9-B0BB5F4D1E77}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{8E47A5CF-CF99-4C53-84E9-B0BB5F4D1E77}"/>
   </bookViews>
   <sheets>
     <sheet name="base" sheetId="1" r:id="rId1"/>
@@ -1084,24 +1084,25 @@
       <sheetName val="P Andreia"/>
       <sheetName val="P ANDREIA NOVO"/>
       <sheetName val="FECHAMENTO MÊS"/>
+      <sheetName val="onde_exportar"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
       <sheetData sheetId="1">
         <row r="2">
           <cell r="H2">
-            <v>426.6</v>
+            <v>3599.4</v>
           </cell>
           <cell r="I2">
-            <v>0</v>
+            <v>1433.45</v>
           </cell>
         </row>
         <row r="3">
           <cell r="H3">
-            <v>1790.88</v>
+            <v>3449.04</v>
           </cell>
           <cell r="I3">
-            <v>2217.0300000000002</v>
+            <v>5400.25</v>
           </cell>
         </row>
         <row r="4">
@@ -1109,53 +1110,54 @@
             <v>0</v>
           </cell>
           <cell r="I4">
-            <v>0</v>
+            <v>90.15</v>
           </cell>
         </row>
         <row r="5">
           <cell r="H5">
-            <v>1573.08</v>
+            <v>3907.32</v>
           </cell>
           <cell r="I5">
-            <v>1985.97</v>
+            <v>5651.21</v>
           </cell>
         </row>
         <row r="6">
           <cell r="H6">
-            <v>1912.32</v>
+            <v>3763.68</v>
           </cell>
           <cell r="I6">
-            <v>1156.7</v>
+            <v>3540.17</v>
           </cell>
         </row>
         <row r="7">
           <cell r="H7">
-            <v>399.96</v>
+            <v>569.04</v>
           </cell>
           <cell r="I7">
-            <v>3061.07</v>
+            <v>7308.46</v>
           </cell>
         </row>
         <row r="8">
           <cell r="H8">
-            <v>1280.4000000000001</v>
+            <v>2042.52</v>
           </cell>
           <cell r="I8">
-            <v>2546.92</v>
+            <v>2749.09</v>
           </cell>
         </row>
         <row r="9">
           <cell r="H9">
-            <v>2584.08</v>
+            <v>4661.88</v>
           </cell>
           <cell r="I9">
-            <v>5163.12</v>
+            <v>9478.2999999999993</v>
           </cell>
         </row>
       </sheetData>
       <sheetData sheetId="2"/>
       <sheetData sheetId="3"/>
       <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2002,15 +2004,15 @@
       </c>
       <c r="E18" s="30">
         <f>'[1]P Eliane'!$I$3</f>
-        <v>2217.0300000000002</v>
+        <v>5400.25</v>
       </c>
       <c r="F18" s="30">
         <f>'[1]P Eliane'!$H$3</f>
-        <v>1790.88</v>
+        <v>3449.04</v>
       </c>
       <c r="G18" s="30">
         <f t="shared" ref="G18:G26" si="1">SUM(F18,C18)</f>
-        <v>3759.7200000000003</v>
+        <v>5417.88</v>
       </c>
       <c r="H18" s="8"/>
       <c r="J18" s="6"/>
@@ -2034,15 +2036,15 @@
       </c>
       <c r="E19" s="30">
         <f>'[1]P Eliane'!$I$7</f>
-        <v>3061.07</v>
+        <v>7308.46</v>
       </c>
       <c r="F19" s="30">
         <f>'[1]P Eliane'!$H$7</f>
-        <v>399.96</v>
+        <v>569.04</v>
       </c>
       <c r="G19" s="30">
         <f t="shared" si="1"/>
-        <v>3212.67</v>
+        <v>3381.75</v>
       </c>
       <c r="H19" s="8"/>
       <c r="J19" s="6"/>
@@ -2066,15 +2068,15 @@
       </c>
       <c r="E20" s="30">
         <f>'[1]P Eliane'!$I$8</f>
-        <v>2546.92</v>
+        <v>2749.09</v>
       </c>
       <c r="F20" s="30">
         <f>'[1]P Eliane'!$H$8</f>
-        <v>1280.4000000000001</v>
+        <v>2042.52</v>
       </c>
       <c r="G20" s="30">
         <f t="shared" si="1"/>
-        <v>3437.01</v>
+        <v>4199.13</v>
       </c>
       <c r="H20" s="8"/>
       <c r="J20" s="6"/>
@@ -2098,15 +2100,15 @@
       </c>
       <c r="E21" s="30">
         <f>'[1]P Eliane'!$I$9</f>
-        <v>5163.12</v>
+        <v>9478.2999999999993</v>
       </c>
       <c r="F21" s="30">
         <f>'[1]P Eliane'!$H$9</f>
-        <v>2584.08</v>
+        <v>4661.88</v>
       </c>
       <c r="G21" s="30">
         <f t="shared" si="1"/>
-        <v>7349.47</v>
+        <v>9427.27</v>
       </c>
       <c r="H21" s="8"/>
       <c r="J21" s="6"/>
@@ -2130,15 +2132,15 @@
       </c>
       <c r="E22" s="30">
         <f>'[1]P Eliane'!$I$5</f>
-        <v>1985.97</v>
+        <v>5651.21</v>
       </c>
       <c r="F22" s="30">
         <f>'[1]P Eliane'!$H$5</f>
-        <v>1573.08</v>
+        <v>3907.32</v>
       </c>
       <c r="G22" s="30">
         <f t="shared" si="1"/>
-        <v>4618.5599999999995</v>
+        <v>6952.8</v>
       </c>
       <c r="H22" s="8"/>
       <c r="J22" s="6"/>
@@ -2162,15 +2164,15 @@
       </c>
       <c r="E23" s="30">
         <f>'[1]P Eliane'!$I$6</f>
-        <v>1156.7</v>
+        <v>3540.17</v>
       </c>
       <c r="F23" s="30">
         <f>'[1]P Eliane'!$H$6</f>
-        <v>1912.32</v>
+        <v>3763.68</v>
       </c>
       <c r="G23" s="30">
         <f t="shared" si="1"/>
-        <v>8403.4600000000009</v>
+        <v>10254.82</v>
       </c>
       <c r="H23" s="8"/>
       <c r="J23" s="6"/>
@@ -2194,7 +2196,7 @@
       </c>
       <c r="E24" s="30">
         <f>'[1]P Eliane'!$I$4</f>
-        <v>0</v>
+        <v>90.15</v>
       </c>
       <c r="F24" s="30">
         <f>'[1]P Eliane'!$H$4</f>
@@ -2226,15 +2228,15 @@
       </c>
       <c r="E25" s="30">
         <f>'[1]P Eliane'!$I$2</f>
-        <v>0</v>
+        <v>1433.45</v>
       </c>
       <c r="F25" s="30">
         <f>'[1]P Eliane'!$H$2</f>
-        <v>426.6</v>
+        <v>3599.4</v>
       </c>
       <c r="G25" s="30">
         <f t="shared" si="1"/>
-        <v>4905.5200000000004</v>
+        <v>8078.32</v>
       </c>
       <c r="H25" s="8"/>
       <c r="J25" s="6"/>
@@ -2281,15 +2283,15 @@
       </c>
       <c r="E27" s="38">
         <f>SUM(E18:E25)</f>
-        <v>16130.81</v>
+        <v>35651.079999999994</v>
       </c>
       <c r="F27" s="31">
         <f>SUM(F18:F25)</f>
-        <v>9967.32</v>
+        <v>21992.880000000001</v>
       </c>
       <c r="G27" s="31">
         <f>SUM(G18:G25)</f>
-        <v>37367.46</v>
+        <v>49393.020000000004</v>
       </c>
       <c r="H27" s="8"/>
       <c r="J27" s="6"/>
@@ -3100,6 +3102,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="671776c5-29b2-438f-93e2-4095a3782164" xsi:nil="true"/>
@@ -3108,15 +3119,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3139,6 +3141,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{073DE036-2C71-4DAE-AACC-05156901298A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FFF36B7-B82C-4297-AD0D-C696E2E30F28}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -3153,12 +3163,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{073DE036-2C71-4DAE-AACC-05156901298A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>